<commit_message>
Update UI new page
</commit_message>
<xml_diff>
--- a/aspnet-core/src/HRMv2.Web.Host/wwwroot/template/Export-ReportSalary.xlsx
+++ b/aspnet-core/src/HRMv2.Web.Host/wwwroot/template/Export-ReportSalary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5072A431-A54B-443F-896A-2F03E509C85A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F92517E-57C6-4365-8B0A-AD04979240B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1224" yWindow="1188" windowWidth="21600" windowHeight="11232" xr2:uid="{15B0A3F3-DF1A-4DF6-A8BB-08B5516BAA62}"/>
+    <workbookView xWindow="32145" yWindow="4035" windowWidth="22635" windowHeight="10605" xr2:uid="{15B0A3F3-DF1A-4DF6-A8BB-08B5516BAA62}"/>
   </bookViews>
   <sheets>
     <sheet name="Employee" sheetId="1" r:id="rId1"/>
@@ -82,10 +82,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-  </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -119,6 +116,14 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -140,19 +145,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -470,39 +474,58 @@
   <dimension ref="A1:O1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.6640625" customWidth="1"/>
-    <col min="2" max="3" width="23.88671875" style="2" customWidth="1"/>
-    <col min="4" max="6" width="25.88671875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="29.33203125" customWidth="1"/>
-    <col min="8" max="8" width="29" customWidth="1"/>
-    <col min="9" max="9" width="27.5546875" customWidth="1"/>
-    <col min="10" max="10" width="19" customWidth="1"/>
-    <col min="11" max="11" width="15.5546875" customWidth="1"/>
-    <col min="12" max="12" width="44.6640625" customWidth="1"/>
-    <col min="13" max="13" width="36.109375" customWidth="1"/>
-    <col min="14" max="14" width="17.44140625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="33" customWidth="1"/>
+    <col min="1" max="1" width="14.5546875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="43.88671875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="23.88671875" style="6" customWidth="1"/>
+    <col min="4" max="5" width="21.5546875" style="5" customWidth="1"/>
+    <col min="6" max="6" width="21" style="5" customWidth="1"/>
+    <col min="7" max="7" width="21.33203125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="20.33203125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="21.109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="21.5546875" style="5" customWidth="1"/>
+    <col min="11" max="11" width="21.44140625" style="5" customWidth="1"/>
+    <col min="12" max="12" width="20.88671875" style="5" customWidth="1"/>
+    <col min="13" max="13" width="22.44140625" style="5" customWidth="1"/>
+    <col min="14" max="14" width="21.44140625" style="5" customWidth="1"/>
+    <col min="15" max="15" width="21" style="5" customWidth="1"/>
+    <col min="16" max="16" width="21.109375" style="5" customWidth="1"/>
+    <col min="17" max="17" width="21" style="5" customWidth="1"/>
+    <col min="18" max="18" width="21.6640625" style="5" customWidth="1"/>
+    <col min="19" max="19" width="21.109375" style="5" customWidth="1"/>
+    <col min="20" max="20" width="21" style="5" customWidth="1"/>
+    <col min="21" max="21" width="20.88671875" style="5" customWidth="1"/>
+    <col min="22" max="22" width="21.21875" style="5" customWidth="1"/>
+    <col min="23" max="23" width="21" style="5" customWidth="1"/>
+    <col min="24" max="24" width="20.77734375" style="5" customWidth="1"/>
+    <col min="25" max="25" width="21.109375" style="5" customWidth="1"/>
+    <col min="26" max="26" width="21" style="5" customWidth="1"/>
+    <col min="27" max="27" width="20.88671875" style="5" customWidth="1"/>
+    <col min="28" max="28" width="21.21875" style="5" customWidth="1"/>
+    <col min="29" max="29" width="21" style="5" customWidth="1"/>
+    <col min="30" max="31" width="21.44140625" style="5" customWidth="1"/>
+    <col min="32" max="32" width="20.88671875" style="5" customWidth="1"/>
+    <col min="33" max="33" width="21.109375" style="5" customWidth="1"/>
+    <col min="34" max="34" width="21.44140625" style="5" customWidth="1"/>
+    <col min="35" max="35" width="21" style="5" customWidth="1"/>
+    <col min="36" max="16384" width="8.88671875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="4" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:15" s="3" customFormat="1" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="7"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -538,18 +561,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -557,7 +580,7 @@
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -565,7 +588,7 @@
       <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>